<commit_message>
Ell: Organizando algumas figuras e códigos. Adicionando rarefação
</commit_message>
<xml_diff>
--- a/res/tabela de habitat_pt.xlsx
+++ b/res/tabela de habitat_pt.xlsx
@@ -1,27 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="tabela_final" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="tabela_final" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="600">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="600">
   <si>
     <t xml:space="preserve">Variable</t>
   </si>
@@ -1826,11 +1820,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1839,40 +1833,27 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFFC000"/>
       <name val="Calibri"/>
       <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1890,7 +1871,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -1898,81 +1879,48 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="general" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-  </cellStyleXfs>
-  <cellXfs count="10">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="left" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="left" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
+    <xf numFmtId="164" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="general" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="general" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="general" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="general" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="false" hidden="false"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment textRotation="0" horizontal="general" vertical="bottom" indent="0"/>
+      <protection hidden="0" locked="0"/>
     </xf>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -2264,14 +2212,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
-  <sheetFormatPr defaultColWidth="10.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2321,7 +2269,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>16</v>
       </c>
@@ -2371,7 +2319,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>32</v>
       </c>
@@ -2421,7 +2369,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>48</v>
       </c>
@@ -2471,7 +2419,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>61</v>
       </c>
@@ -2521,7 +2469,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>77</v>
       </c>
@@ -2571,7 +2519,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" ht="15" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>93</v>
       </c>
@@ -2621,7 +2569,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" ht="15" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>109</v>
       </c>
@@ -2671,7 +2619,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>123</v>
       </c>
@@ -2721,7 +2669,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" ht="15" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>138</v>
       </c>
@@ -2771,7 +2719,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" ht="15" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>154</v>
       </c>
@@ -2821,7 +2769,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>170</v>
       </c>
@@ -2871,7 +2819,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" ht="15" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>186</v>
       </c>
@@ -2921,7 +2869,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" ht="15" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>202</v>
       </c>
@@ -2971,7 +2919,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" ht="15" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>217</v>
       </c>
@@ -3021,7 +2969,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" ht="15" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>231</v>
       </c>
@@ -3071,7 +3019,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" ht="15" customHeight="1">
       <c r="A17" s="1" t="s">
         <v>233</v>
       </c>
@@ -3121,7 +3069,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" ht="15" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>234</v>
       </c>
@@ -3171,7 +3119,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" ht="15" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>240</v>
       </c>
@@ -3221,7 +3169,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" ht="15" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>245</v>
       </c>
@@ -3271,7 +3219,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" ht="15" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>256</v>
       </c>
@@ -3321,7 +3269,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" ht="15" customHeight="1">
       <c r="A22" s="1" t="s">
         <v>271</v>
       </c>
@@ -3371,7 +3319,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" ht="15" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>278</v>
       </c>
@@ -3421,7 +3369,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" ht="15" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>289</v>
       </c>
@@ -3471,7 +3419,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" ht="15" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>297</v>
       </c>
@@ -3522,28 +3470,28 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.597222222222222" bottom="0.597222222222222" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
+    <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P36"/>
-  <sheetFormatPr defaultColWidth="10.54296875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="1" width="14.42"/>
+    <col min="12" max="12" width="14.42" hidden="false" outlineLevel="0" customWidth="1"/>
+    <col min="13" max="13" width="14.42" hidden="false" outlineLevel="0" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" ht="13.5" customHeight="1">
       <c r="B1" s="2" t="s">
         <v>311</v>
       </c>
@@ -3564,7 +3512,7 @@
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
     </row>
-    <row r="2" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" ht="13.5" customHeight="1">
       <c r="B2" s="1" t="s">
         <v>313</v>
       </c>
@@ -3611,23 +3559,23 @@
         <v>327</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
+    <row r="3" ht="13.5" customHeight="1">
+      <c r="A3" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="B3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="5"/>
-      <c r="K3" s="5"/>
-      <c r="L3" s="5"/>
-      <c r="M3" s="5"/>
-      <c r="N3" s="5"/>
-      <c r="O3" s="5"/>
-      <c r="P3" s="5"/>
-    </row>
-    <row r="4" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+    </row>
+    <row r="4" ht="13.5" customHeight="1">
       <c r="A4" s="1" t="s">
         <v>329</v>
       </c>
@@ -3677,7 +3625,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" ht="13.5" customHeight="1">
       <c r="A5" s="1" t="s">
         <v>345</v>
       </c>
@@ -3727,7 +3675,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" ht="13.5" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>361</v>
       </c>
@@ -3749,35 +3697,35 @@
       <c r="G6" s="1" t="s">
         <v>367</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="4" t="s">
         <v>368</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="J6" s="5" t="s">
+      <c r="J6" s="4" t="s">
         <v>370</v>
       </c>
-      <c r="K6" s="5" t="s">
+      <c r="K6" s="4" t="s">
         <v>371</v>
       </c>
-      <c r="L6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="5" t="s">
+      <c r="L6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="4" t="s">
         <v>372</v>
       </c>
-      <c r="N6" s="5" t="s">
+      <c r="N6" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="O6" s="6" t="s">
+      <c r="O6" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="P6" s="5" t="s">
+      <c r="P6" s="4" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" ht="13.5" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>376</v>
       </c>
@@ -3799,35 +3747,35 @@
       <c r="G7" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="4" t="s">
         <v>383</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="4" t="s">
         <v>384</v>
       </c>
-      <c r="J7" s="5" t="s">
+      <c r="J7" s="4" t="s">
         <v>385</v>
       </c>
-      <c r="K7" s="5" t="s">
+      <c r="K7" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="L7" s="5" t="s">
+      <c r="L7" s="4" t="s">
         <v>387</v>
       </c>
-      <c r="M7" s="5" t="s">
+      <c r="M7" s="4" t="s">
         <v>388</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="N7" s="4" t="s">
         <v>389</v>
       </c>
-      <c r="O7" s="5" t="s">
+      <c r="O7" s="4" t="s">
         <v>390</v>
       </c>
-      <c r="P7" s="5" t="s">
+      <c r="P7" s="4" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" ht="13.5" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>392</v>
       </c>
@@ -3849,35 +3797,35 @@
       <c r="G8" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="4" t="s">
         <v>399</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="4" t="s">
         <v>400</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="4" t="s">
         <v>401</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="K8" s="4" t="s">
         <v>402</v>
       </c>
-      <c r="L8" s="5" t="s">
+      <c r="L8" s="4" t="s">
         <v>403</v>
       </c>
-      <c r="M8" s="5" t="s">
+      <c r="M8" s="4" t="s">
         <v>404</v>
       </c>
-      <c r="N8" s="5" t="s">
+      <c r="N8" s="4" t="s">
         <v>405</v>
       </c>
-      <c r="O8" s="5" t="s">
+      <c r="O8" s="4" t="s">
         <v>406</v>
       </c>
-      <c r="P8" s="5" t="s">
+      <c r="P8" s="4" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" ht="13.5" customHeight="1">
       <c r="A9" s="1" t="s">
         <v>408</v>
       </c>
@@ -3899,51 +3847,51 @@
       <c r="G9" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="4" t="s">
         <v>415</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="4" t="s">
         <v>416</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="J9" s="4" t="s">
         <v>417</v>
       </c>
-      <c r="K9" s="5" t="s">
+      <c r="K9" s="4" t="s">
         <v>418</v>
       </c>
-      <c r="L9" s="5" t="s">
+      <c r="L9" s="4" t="s">
         <v>419</v>
       </c>
-      <c r="M9" s="5" t="s">
+      <c r="M9" s="4" t="s">
         <v>420</v>
       </c>
-      <c r="N9" s="5" t="s">
+      <c r="N9" s="4" t="s">
         <v>421</v>
       </c>
-      <c r="O9" s="5" t="s">
+      <c r="O9" s="4" t="s">
         <v>422</v>
       </c>
-      <c r="P9" s="5" t="s">
+      <c r="P9" s="4" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+    <row r="10" ht="13.5" customHeight="1">
+      <c r="A10" s="2" t="s">
         <v>424</v>
       </c>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="H10" s="5"/>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-      <c r="K10" s="5"/>
-      <c r="L10" s="5"/>
-      <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
-      <c r="P10" s="5"/>
-    </row>
-    <row r="11" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
+      <c r="J10" s="4"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="4"/>
+    </row>
+    <row r="11" ht="13.5" customHeight="1">
       <c r="A11" s="1" t="s">
         <v>425</v>
       </c>
@@ -3965,35 +3913,35 @@
       <c r="G11" s="1" t="s">
         <v>429</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="4" t="s">
         <v>117</v>
       </c>
-      <c r="J11" s="5" t="s">
+      <c r="J11" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="K11" s="5" t="s">
+      <c r="K11" s="4" t="s">
         <v>119</v>
       </c>
-      <c r="L11" s="5" t="s">
+      <c r="L11" s="4" t="s">
         <v>118</v>
       </c>
-      <c r="M11" s="5" t="s">
+      <c r="M11" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="N11" s="5" t="s">
+      <c r="N11" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="O11" s="5" t="s">
+      <c r="O11" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="P11" s="5" t="s">
+      <c r="P11" s="4" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" ht="13.5" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>430</v>
       </c>
@@ -4015,35 +3963,35 @@
       <c r="G12" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="4" t="s">
         <v>437</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="4" t="s">
         <v>438</v>
       </c>
-      <c r="J12" s="5" t="s">
+      <c r="J12" s="4" t="s">
         <v>439</v>
       </c>
-      <c r="K12" s="5" t="s">
+      <c r="K12" s="4" t="s">
         <v>440</v>
       </c>
-      <c r="L12" s="5" t="s">
+      <c r="L12" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="M12" s="5" t="s">
+      <c r="M12" s="4" t="s">
         <v>441</v>
       </c>
-      <c r="N12" s="5" t="s">
+      <c r="N12" s="4" t="s">
         <v>134</v>
       </c>
-      <c r="O12" s="5" t="s">
+      <c r="O12" s="4" t="s">
         <v>442</v>
       </c>
-      <c r="P12" s="5" t="s">
+      <c r="P12" s="4" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" ht="13.5" customHeight="1">
       <c r="A13" s="1" t="s">
         <v>444</v>
       </c>
@@ -4065,35 +4013,35 @@
       <c r="G13" s="1" t="s">
         <v>450</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="4" t="s">
         <v>451</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="4" t="s">
         <v>452</v>
       </c>
-      <c r="J13" s="5" t="s">
+      <c r="J13" s="4" t="s">
         <v>453</v>
       </c>
-      <c r="K13" s="5" t="s">
+      <c r="K13" s="4" t="s">
         <v>454</v>
       </c>
-      <c r="L13" s="7" t="s">
+      <c r="L13" s="6" t="s">
         <v>455</v>
       </c>
-      <c r="M13" s="7" t="s">
+      <c r="M13" s="6" t="s">
         <v>456</v>
       </c>
-      <c r="N13" s="5" t="s">
+      <c r="N13" s="4" t="s">
         <v>457</v>
       </c>
-      <c r="O13" s="5" t="s">
+      <c r="O13" s="4" t="s">
         <v>458</v>
       </c>
-      <c r="P13" s="5" t="s">
+      <c r="P13" s="4" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" ht="13.5" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>460</v>
       </c>
@@ -4115,35 +4063,35 @@
       <c r="G14" s="1" t="s">
         <v>466</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="4" t="s">
         <v>467</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="4" t="s">
         <v>468</v>
       </c>
-      <c r="J14" s="5" t="s">
+      <c r="J14" s="4" t="s">
         <v>469</v>
       </c>
-      <c r="K14" s="5" t="s">
+      <c r="K14" s="4" t="s">
         <v>470</v>
       </c>
-      <c r="L14" s="5" t="s">
+      <c r="L14" s="4" t="s">
         <v>471</v>
       </c>
-      <c r="M14" s="5" t="s">
+      <c r="M14" s="4" t="s">
         <v>472</v>
       </c>
-      <c r="N14" s="5" t="s">
+      <c r="N14" s="4" t="s">
         <v>473</v>
       </c>
-      <c r="O14" s="5" t="s">
+      <c r="O14" s="4" t="s">
         <v>474</v>
       </c>
-      <c r="P14" s="5" t="s">
+      <c r="P14" s="4" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" ht="13.5" customHeight="1">
       <c r="A15" s="1" t="s">
         <v>475</v>
       </c>
@@ -4177,10 +4125,10 @@
       <c r="K15" s="1" t="s">
         <v>485</v>
       </c>
-      <c r="L15" s="8" t="s">
+      <c r="L15" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="M15" s="8" t="s">
+      <c r="M15" s="7" t="s">
         <v>486</v>
       </c>
       <c r="N15" s="1" t="s">
@@ -4193,7 +4141,7 @@
         <v>489</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" ht="13.5" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>490</v>
       </c>
@@ -4243,30 +4191,30 @@
         <v>505</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
+    <row r="17" ht="13.5" customHeight="1">
+      <c r="A17" s="2" t="s">
         <v>506</v>
       </c>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="H17" s="5"/>
-      <c r="I17" s="5"/>
-      <c r="J17" s="5"/>
-      <c r="K17" s="5"/>
-      <c r="L17" s="5"/>
-      <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
-      <c r="P17" s="5"/>
-    </row>
-    <row r="18" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="H17" s="4"/>
+      <c r="I17" s="4"/>
+      <c r="J17" s="4"/>
+      <c r="K17" s="4"/>
+      <c r="L17" s="4"/>
+      <c r="M17" s="4"/>
+      <c r="N17" s="4"/>
+      <c r="O17" s="4"/>
+      <c r="P17" s="4"/>
+    </row>
+    <row r="18" ht="13.5" customHeight="1">
       <c r="A18" s="1" t="s">
         <v>507</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="B18" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="8" t="s">
         <v>203</v>
       </c>
       <c r="D18" s="1" t="s">
@@ -4281,35 +4229,35 @@
       <c r="G18" s="1" t="s">
         <v>510</v>
       </c>
-      <c r="H18" s="5" t="s">
+      <c r="H18" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="I18" s="5" t="s">
+      <c r="I18" s="4" t="s">
         <v>511</v>
       </c>
-      <c r="J18" s="5" t="s">
+      <c r="J18" s="4" t="s">
         <v>512</v>
       </c>
-      <c r="K18" s="5" t="s">
+      <c r="K18" s="4" t="s">
         <v>513</v>
       </c>
-      <c r="L18" s="5" t="s">
+      <c r="L18" s="4" t="s">
         <v>514</v>
       </c>
-      <c r="M18" s="5" t="s">
+      <c r="M18" s="4" t="s">
         <v>515</v>
       </c>
-      <c r="N18" s="5" t="s">
+      <c r="N18" s="4" t="s">
         <v>516</v>
       </c>
-      <c r="O18" s="5" t="s">
+      <c r="O18" s="4" t="s">
         <v>517</v>
       </c>
-      <c r="P18" s="5" t="s">
+      <c r="P18" s="4" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" ht="13.5" customHeight="1">
       <c r="A19" s="1" t="s">
         <v>519</v>
       </c>
@@ -4331,35 +4279,35 @@
       <c r="G19" s="1" t="s">
         <v>522</v>
       </c>
-      <c r="H19" s="5" t="s">
+      <c r="H19" s="4" t="s">
         <v>222</v>
       </c>
-      <c r="I19" s="5" t="s">
+      <c r="I19" s="4" t="s">
         <v>523</v>
       </c>
-      <c r="J19" s="6" t="s">
+      <c r="J19" s="5" t="s">
         <v>524</v>
       </c>
-      <c r="K19" s="6" t="s">
+      <c r="K19" s="5" t="s">
         <v>525</v>
       </c>
-      <c r="L19" s="5" t="s">
+      <c r="L19" s="4" t="s">
         <v>526</v>
       </c>
-      <c r="M19" s="5" t="s">
+      <c r="M19" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="N19" s="5" t="s">
+      <c r="N19" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="O19" s="6" t="s">
+      <c r="O19" s="5" t="s">
         <v>528</v>
       </c>
-      <c r="P19" s="5" t="s">
+      <c r="P19" s="4" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" ht="13.5" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>530</v>
       </c>
@@ -4381,35 +4329,35 @@
       <c r="G20" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="5" t="s">
+      <c r="H20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="K20" s="5" t="s">
+      <c r="K20" s="4" t="s">
         <v>531</v>
       </c>
-      <c r="L20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="5" t="s">
+      <c r="L20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="4" t="s">
         <v>531</v>
       </c>
-      <c r="O20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="13.5" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>532</v>
       </c>
@@ -4431,51 +4379,51 @@
       <c r="G21" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M21" s="5" t="s">
+      <c r="H21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="4" t="s">
         <v>531</v>
       </c>
-      <c r="N21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
+      <c r="N21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P21" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="13.5" customHeight="1">
+      <c r="A22" s="2" t="s">
         <v>533</v>
       </c>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="H22" s="5"/>
-      <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
-      <c r="K22" s="5"/>
-      <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
-      <c r="P22" s="5"/>
-    </row>
-    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="H22" s="4"/>
+      <c r="I22" s="4"/>
+      <c r="J22" s="4"/>
+      <c r="K22" s="4"/>
+      <c r="L22" s="4"/>
+      <c r="M22" s="4"/>
+      <c r="N22" s="4"/>
+      <c r="O22" s="4"/>
+      <c r="P22" s="4"/>
+    </row>
+    <row r="23" ht="13.5" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>534</v>
       </c>
@@ -4485,47 +4433,47 @@
       <c r="C23" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="D23" s="8" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>536</v>
       </c>
-      <c r="F23" s="9" t="n">
+      <c r="F23" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G23" s="1" t="s">
         <v>517</v>
       </c>
-      <c r="H23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" s="5" t="s">
+      <c r="H23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I23" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="J23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="5" t="s">
+      <c r="J23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="4" t="s">
         <v>537</v>
       </c>
-      <c r="M23" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N23" s="5" t="s">
+      <c r="M23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" s="4" t="s">
         <v>538</v>
       </c>
-      <c r="O23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="13.5" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>539</v>
       </c>
@@ -4541,41 +4489,41 @@
       <c r="E24" s="1" t="s">
         <v>543</v>
       </c>
-      <c r="F24" s="9" t="n">
+      <c r="F24" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G24" s="1" t="s">
         <v>527</v>
       </c>
-      <c r="H24" s="5" t="s">
+      <c r="H24" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="I24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="L24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="I24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="13.5" customHeight="1">
       <c r="A25" s="1" t="s">
         <v>544</v>
       </c>
@@ -4597,35 +4545,35 @@
       <c r="G25" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="H25" s="5" t="s">
+      <c r="H25" s="4" t="s">
         <v>517</v>
       </c>
-      <c r="I25" s="5" t="s">
+      <c r="I25" s="4" t="s">
         <v>549</v>
       </c>
-      <c r="J25" s="5" t="s">
+      <c r="J25" s="4" t="s">
         <v>251</v>
       </c>
-      <c r="K25" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L25" s="5" t="s">
+      <c r="K25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="4" t="s">
         <v>550</v>
       </c>
-      <c r="M25" s="5" t="s">
+      <c r="M25" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="N25" s="5" t="s">
+      <c r="N25" s="4" t="s">
         <v>254</v>
       </c>
-      <c r="O25" s="5" t="s">
+      <c r="O25" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="P25" s="5" t="s">
+      <c r="P25" s="4" t="s">
         <v>551</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" ht="13.5" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>552</v>
       </c>
@@ -4647,35 +4595,35 @@
       <c r="G26" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="H26" s="5" t="s">
+      <c r="H26" s="4" t="s">
         <v>557</v>
       </c>
-      <c r="I26" s="5" t="s">
+      <c r="I26" s="4" t="s">
         <v>558</v>
       </c>
-      <c r="J26" s="5" t="s">
+      <c r="J26" s="4" t="s">
         <v>559</v>
       </c>
-      <c r="K26" s="5" t="s">
+      <c r="K26" s="4" t="s">
         <v>266</v>
       </c>
-      <c r="L26" s="5" t="s">
+      <c r="L26" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="M26" s="5" t="s">
+      <c r="M26" s="4" t="s">
         <v>560</v>
       </c>
-      <c r="N26" s="5" t="s">
+      <c r="N26" s="4" t="s">
         <v>561</v>
       </c>
-      <c r="O26" s="5" t="s">
+      <c r="O26" s="4" t="s">
         <v>562</v>
       </c>
-      <c r="P26" s="5" t="s">
+      <c r="P26" s="4" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" ht="13.5" customHeight="1">
       <c r="A27" s="1" t="s">
         <v>564</v>
       </c>
@@ -4691,41 +4639,41 @@
       <c r="E27" s="1" t="s">
         <v>566</v>
       </c>
-      <c r="F27" s="9" t="n">
+      <c r="F27" s="8" t="n">
         <v>0</v>
       </c>
       <c r="G27" s="1" t="s">
         <v>567</v>
       </c>
-      <c r="H27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="5" t="s">
+      <c r="H27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="L27" s="5" t="s">
+      <c r="L27" s="4" t="s">
         <v>568</v>
       </c>
-      <c r="M27" s="5" t="s">
+      <c r="M27" s="4" t="s">
         <v>535</v>
       </c>
-      <c r="N27" s="5" t="s">
+      <c r="N27" s="4" t="s">
         <v>569</v>
       </c>
-      <c r="O27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="13.5" customHeight="1">
       <c r="A28" s="1" t="s">
         <v>570</v>
       </c>
@@ -4747,35 +4695,35 @@
       <c r="G28" s="1" t="s">
         <v>575</v>
       </c>
-      <c r="H28" s="5" t="s">
+      <c r="H28" s="4" t="s">
         <v>545</v>
       </c>
-      <c r="I28" s="5" t="s">
+      <c r="I28" s="4" t="s">
         <v>576</v>
       </c>
-      <c r="J28" s="5" t="s">
+      <c r="J28" s="4" t="s">
         <v>286</v>
       </c>
-      <c r="K28" s="5" t="s">
+      <c r="K28" s="4" t="s">
         <v>571</v>
       </c>
-      <c r="L28" s="5" t="s">
+      <c r="L28" s="4" t="s">
         <v>517</v>
       </c>
-      <c r="M28" s="5" t="s">
+      <c r="M28" s="4" t="s">
         <v>540</v>
       </c>
-      <c r="N28" s="5" t="s">
+      <c r="N28" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="O28" s="5" t="s">
+      <c r="O28" s="4" t="s">
         <v>577</v>
       </c>
-      <c r="P28" s="5" t="s">
+      <c r="P28" s="4" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" ht="13.5" customHeight="1">
       <c r="A29" s="1" t="s">
         <v>579</v>
       </c>
@@ -4797,35 +4745,35 @@
       <c r="G29" s="1" t="s">
         <v>565</v>
       </c>
-      <c r="H29" s="5" t="s">
+      <c r="H29" s="4" t="s">
         <v>547</v>
       </c>
-      <c r="I29" s="5" t="s">
+      <c r="I29" s="4" t="s">
         <v>253</v>
       </c>
-      <c r="J29" s="5" t="s">
+      <c r="J29" s="4" t="s">
         <v>583</v>
       </c>
-      <c r="K29" s="5" t="s">
+      <c r="K29" s="4" t="s">
         <v>584</v>
       </c>
-      <c r="L29" s="5" t="s">
+      <c r="L29" s="4" t="s">
         <v>527</v>
       </c>
-      <c r="M29" s="5" t="s">
+      <c r="M29" s="4" t="s">
         <v>580</v>
       </c>
-      <c r="N29" s="5" t="s">
+      <c r="N29" s="4" t="s">
         <v>585</v>
       </c>
-      <c r="O29" s="5" t="s">
+      <c r="O29" s="4" t="s">
         <v>545</v>
       </c>
-      <c r="P29" s="5" t="s">
+      <c r="P29" s="4" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" ht="13.5" customHeight="1">
       <c r="A30" s="1" t="s">
         <v>587</v>
       </c>
@@ -4847,37 +4795,37 @@
       <c r="G30" s="1" t="s">
         <v>593</v>
       </c>
-      <c r="H30" s="5" t="s">
+      <c r="H30" s="4" t="s">
         <v>594</v>
       </c>
-      <c r="I30" s="5" t="s">
+      <c r="I30" s="4" t="s">
         <v>595</v>
       </c>
-      <c r="J30" s="5" t="s">
+      <c r="J30" s="4" t="s">
         <v>596</v>
       </c>
-      <c r="K30" s="5" t="s">
+      <c r="K30" s="4" t="s">
         <v>597</v>
       </c>
-      <c r="L30" s="5" t="s">
+      <c r="L30" s="4" t="s">
         <v>569</v>
       </c>
-      <c r="M30" s="5" t="s">
+      <c r="M30" s="4" t="s">
         <v>598</v>
       </c>
-      <c r="N30" s="5" t="s">
+      <c r="N30" s="4" t="s">
         <v>309</v>
       </c>
-      <c r="O30" s="5" t="s">
+      <c r="O30" s="4" t="s">
         <v>538</v>
       </c>
-      <c r="P30" s="5" t="s">
+      <c r="P30" s="4" t="s">
         <v>599</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="L36" s="9"/>
-      <c r="M36" s="9"/>
+    <row r="36" ht="13.5" customHeight="1">
+      <c r="L36" s="8"/>
+      <c r="M36" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -4886,12 +4834,11 @@
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A22:C22"/>
   </mergeCells>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPágina &amp;P</oddFooter>
+  <headerFooter differentOddEven="0" differentFirst="0" scaleWithDoc="0" alignWithMargins="0">
+    <oddHeader>&amp;L&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;Kffffff&amp;A&amp;R</oddHeader>
+    <oddFooter>&amp;L&amp;C&amp;"Times New Roman,Normal"&amp;12&amp;KffffffPágina &amp;P&amp;R</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>